<commit_message>
Aggiornamento incrementale DB e Top 15 📈
</commit_message>
<xml_diff>
--- a/Top_15_Live.xlsx
+++ b/Top_15_Live.xlsx
@@ -499,88 +499,88 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>46238</v>
+        <v>46325</v>
       </c>
       <c r="D3" t="n">
         <v>100</v>
       </c>
       <c r="E3" t="n">
-        <v>13.17</v>
+        <v>14.24</v>
       </c>
       <c r="F3" t="n">
-        <v>167.38</v>
+        <v>1150.89</v>
       </c>
       <c r="G3" t="n">
-        <v>12.31</v>
+        <v>5.47</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46240</v>
+        <v>46238</v>
       </c>
       <c r="D4" t="n">
         <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>12.01</v>
+        <v>13.17</v>
       </c>
       <c r="F4" t="n">
-        <v>55.1</v>
+        <v>167.38</v>
       </c>
       <c r="G4" t="n">
-        <v>8.75</v>
+        <v>12.31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>FOX</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>46304</v>
+        <v>46240</v>
       </c>
       <c r="D5" t="n">
         <v>100</v>
       </c>
       <c r="E5" t="n">
-        <v>11.18</v>
+        <v>12.01</v>
       </c>
       <c r="F5" t="n">
-        <v>1028.84</v>
+        <v>55.1</v>
       </c>
       <c r="G5" t="n">
-        <v>7.8</v>
+        <v>8.75</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -589,289 +589,289 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46265</v>
+        <v>46304</v>
       </c>
       <c r="D6" t="n">
         <v>100</v>
       </c>
       <c r="E6" t="n">
-        <v>11.06</v>
+        <v>11.18</v>
       </c>
       <c r="F6" t="n">
-        <v>37.28</v>
+        <v>1028.84</v>
       </c>
       <c r="G6" t="n">
-        <v>5.68</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46240</v>
+        <v>46265</v>
       </c>
       <c r="D7" t="n">
         <v>100</v>
       </c>
       <c r="E7" t="n">
-        <v>10.75</v>
+        <v>11.06</v>
       </c>
       <c r="F7" t="n">
-        <v>61.52</v>
+        <v>37.28</v>
       </c>
       <c r="G7" t="n">
-        <v>9.77</v>
+        <v>5.68</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>FOXA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>46251</v>
+        <v>46240</v>
       </c>
       <c r="D8" t="n">
         <v>100</v>
       </c>
       <c r="E8" t="n">
-        <v>10.23</v>
+        <v>10.75</v>
       </c>
       <c r="F8" t="n">
-        <v>1786.85</v>
+        <v>61.52</v>
       </c>
       <c r="G8" t="n">
-        <v>10.03</v>
+        <v>9.77</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADM</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>46238</v>
+        <v>46251</v>
       </c>
       <c r="D9" t="n">
         <v>100</v>
       </c>
       <c r="E9" t="n">
-        <v>9.109999999999999</v>
+        <v>10.23</v>
       </c>
       <c r="F9" t="n">
-        <v>79.37</v>
+        <v>1786.85</v>
       </c>
       <c r="G9" t="n">
-        <v>15.78</v>
+        <v>8.859999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>ADM</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46311</v>
+        <v>46238</v>
       </c>
       <c r="D10" t="n">
         <v>100</v>
       </c>
       <c r="E10" t="n">
-        <v>8.19</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>229.68</v>
+        <v>79.37</v>
       </c>
       <c r="G10" t="n">
-        <v>17.45</v>
+        <v>15.78</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TSCO</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>46240</v>
+        <v>46325</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
       </c>
       <c r="E11" t="n">
-        <v>7.41</v>
+        <v>8.99</v>
       </c>
       <c r="F11" t="n">
-        <v>33.86</v>
+        <v>170.68</v>
       </c>
       <c r="G11" t="n">
-        <v>12.31</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BF-B</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>46267</v>
+        <v>46311</v>
       </c>
       <c r="D12" t="n">
         <v>100</v>
       </c>
       <c r="E12" t="n">
-        <v>5.16</v>
+        <v>8.19</v>
       </c>
       <c r="F12" t="n">
-        <v>27.15</v>
+        <v>229.68</v>
       </c>
       <c r="G12" t="n">
-        <v>17.72</v>
+        <v>17.45</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RMD</t>
+          <t>TSCO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>46247</v>
+        <v>46240</v>
       </c>
       <c r="D13" t="n">
         <v>100</v>
       </c>
       <c r="E13" t="n">
-        <v>4.89</v>
+        <v>7.41</v>
       </c>
       <c r="F13" t="n">
-        <v>226.09</v>
+        <v>33.86</v>
       </c>
       <c r="G13" t="n">
-        <v>21.53</v>
+        <v>12.31</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LH</t>
+          <t>BF-B</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>46239</v>
+        <v>46267</v>
       </c>
       <c r="D14" t="n">
         <v>100</v>
       </c>
       <c r="E14" t="n">
-        <v>4.89</v>
+        <v>5.16</v>
       </c>
       <c r="F14" t="n">
-        <v>313.29</v>
+        <v>27.15</v>
       </c>
       <c r="G14" t="n">
-        <v>21.5</v>
+        <v>17.72</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>RMD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>46318</v>
+        <v>46247</v>
       </c>
       <c r="D15" t="n">
         <v>100</v>
       </c>
       <c r="E15" t="n">
-        <v>4.17</v>
+        <v>4.89</v>
       </c>
       <c r="F15" t="n">
-        <v>343.67</v>
+        <v>226.09</v>
       </c>
       <c r="G15" t="n">
-        <v>18.55</v>
+        <v>7.34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>RMD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>46289</v>
+        <v>46325</v>
       </c>
       <c r="D16" t="n">
         <v>100</v>
       </c>
       <c r="E16" t="n">
-        <v>3.99</v>
+        <v>4.53</v>
       </c>
       <c r="F16" t="n">
-        <v>100.57</v>
+        <v>229.94</v>
       </c>
       <c r="G16" t="n">
-        <v>20.86</v>
+        <v>19.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>